<commit_message>
Simplify wording in README and workbook notes
</commit_message>
<xml_diff>
--- a/deliverables/premium_screen_model.xlsx
+++ b/deliverables/premium_screen_model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saathvikmaheshuni/premium-screen-investment-model/deliverables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB06A2D-588E-A542-9534-01F0AD3BF5AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D4DE9F6-E3D8-A241-8E67-2D7AFDDD7A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -273,7 +273,7 @@
     <t>Premium projection and sound system per screen</t>
   </si>
   <si>
-    <t>Proxy: IMAX's average revenue per new system installed in 2025 (section B). Applied in every scenario whatever the deal type; under a traditional JRSA, IMAX carries most of this cost, so the downside (blended JRSA share plus full equipment cost) is conservative.</t>
+    <t>Proxy: IMAX's average revenue per new system installed in 2025 (section B). Used in every scenario, whatever the deal type. In a traditional JRSA, IMAX pays for most of this, so the downside (blended JRSA share plus the full equipment cost) is on the cautious side.</t>
   </si>
   <si>
     <t>Auditorium construction per screen (screen wall, sound, seating, structure)</t>
@@ -327,7 +327,7 @@
     <t>Cash tax rate on incremental profit</t>
   </si>
   <si>
-    <t>AMC's federal NOLs (section A) shelter profit over the 10-year window. Raise to test a taxpaying owner; years with a tax loss are assumed to offset other taxable income.</t>
+    <t>AMC's federal NOLs (section A) cover the profit for all 10 years, so there is no cash tax. Raise this to test an owner that pays tax. Years with a tax loss are assumed to offset other taxable income.</t>
   </si>
   <si>
     <t>Depreciation life of the conversion</t>
@@ -636,22 +636,22 @@
     <t>Model checks</t>
   </si>
   <si>
-    <t>What drives the answer</t>
-  </si>
-  <si>
-    <t>1. Attendance uplift and cannibalization decide the result. Only net new patrons add food and beverage profit, and every extra ticket on the converted screen pays film rent and the partner's share.</t>
+    <t>What the result depends on</t>
+  </si>
+  <si>
+    <t>1. Attendance uplift and cannibalization matter most. Only net new patrons add food and beverage profit, and every extra ticket on the converted screen pays film rent and the partner's share.</t>
   </si>
   <si>
     <t>2. The partner's share applies to the whole screen's box office, including tickets the screen sold before conversion, so better deal terms raise NPV directly.</t>
   </si>
   <si>
-    <t>3. A-List subscribers book premium formats at no extra cost, so a higher subscriber mix erodes the surcharge.</t>
-  </si>
-  <si>
-    <t>4. Results depend on a slate of films made for premium formats. A weak year cuts both uplift and surcharge.</t>
-  </si>
-  <si>
-    <t>5. Construction overruns and weeks closed hit the investment up front, before any uplift arrives.</t>
+    <t>3. A-List subscribers book premium formats at no extra cost, so the more A-List subscribers there are, the less surcharge the screen collects.</t>
+  </si>
+  <si>
+    <t>4. The results need enough films made for premium formats. A weak year for those films lowers both the uplift and the surcharge.</t>
+  </si>
+  <si>
+    <t>5. Construction overruns and the weeks the screen is closed both cost money in year 0, before any extra attendance comes in.</t>
   </si>
   <si>
     <t>Checks: recompute the results a second way with Excel's own functions</t>
@@ -1107,7 +1107,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-3B8E-154A-AE03-B1EC43B50DC5}"/>
+                <c16:uniqueId val="{00000001-BDDF-1B42-92A9-7AF92AC8BDE3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1185,7 +1185,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-3B8E-154A-AE03-B1EC43B50DC5}"/>
+              <c16:uniqueId val="{00000002-BDDF-1B42-92A9-7AF92AC8BDE3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1510,7 +1510,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-497A-8D44-A36D-604E9720EF5D}"/>
+              <c16:uniqueId val="{00000000-15D0-4D41-A15B-D26FAB540173}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1596,7 +1596,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-497A-8D44-A36D-604E9720EF5D}"/>
+              <c16:uniqueId val="{00000001-15D0-4D41-A15B-D26FAB540173}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1682,7 +1682,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-497A-8D44-A36D-604E9720EF5D}"/>
+              <c16:uniqueId val="{00000002-15D0-4D41-A15B-D26FAB540173}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3954,7 +3954,7 @@
       </c>
       <c r="F29" s="51" t="str">
         <f>IF(Inputs!G40="","",Inputs!G40)</f>
-        <v>Proxy: IMAX's average revenue per new system installed in 2025 (section B). Applied in every scenario whatever the deal type; under a traditional JRSA, IMAX carries most of this cost, so the downside (blended JRSA share plus full equipment cost) is conservative.</v>
+        <v>Proxy: IMAX's average revenue per new system installed in 2025 (section B). Used in every scenario, whatever the deal type. In a traditional JRSA, IMAX pays for most of this, so the downside (blended JRSA share plus the full equipment cost) is on the cautious side.</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -4188,7 +4188,7 @@
       </c>
       <c r="F38" s="51" t="str">
         <f>IF(Inputs!G49="","",Inputs!G49)</f>
-        <v>AMC's federal NOLs (section A) shelter profit over the 10-year window. Raise to test a taxpaying owner; years with a tax loss are assumed to offset other taxable income.</v>
+        <v>AMC's federal NOLs (section A) cover the profit for all 10 years, so there is no cash tax. Raise this to test an owner that pays tax. Years with a tax loss are assumed to offset other taxable income.</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>